<commit_message>
big cleanup of files
</commit_message>
<xml_diff>
--- a/00_metadata/surfacewater_metadata.xlsx
+++ b/00_metadata/surfacewater_metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/margaretswift/Documents/03 Science/00 Research - Active/Ecosphere Waterholes/eco-kaza-water-ele/00_metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18FC3762-CD22-1F4A-B4E0-C3137BA7DAFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67BBB7C1-35AA-A543-9143-BA695E2BE4D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29400" yWindow="-7880" windowWidth="38400" windowHeight="21100" activeTab="4" xr2:uid="{36B2674D-5574-5749-ABD1-0B06D0B52360}"/>
+    <workbookView xWindow="29400" yWindow="-7880" windowWidth="19340" windowHeight="21100" xr2:uid="{36B2674D-5574-5749-ABD1-0B06D0B52360}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -18,13 +18,14 @@
     <sheet name="MWF_sizes_HY" sheetId="2" r:id="rId3"/>
     <sheet name="ESW_sizes_HY" sheetId="4" r:id="rId4"/>
     <sheet name="ESW_sizes_SIZ" sheetId="5" r:id="rId5"/>
+    <sheet name="AOI_Rasters" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="106">
   <si>
     <t>Data location</t>
   </si>
@@ -309,6 +310,39 @@
   </si>
   <si>
     <t>https://www.hydroshare.org/resource/5b04074877b24501ab3c69813efc6bc3/</t>
+  </si>
+  <si>
+    <t>/01_data/surfacewater/raw/AOI_rasters</t>
+  </si>
+  <si>
+    <t>Rasters of surface water within AOI</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>UTM x coordinate</t>
+  </si>
+  <si>
+    <t>UTM y coordinate</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>frequency</t>
+  </si>
+  <si>
+    <t>recurrence</t>
+  </si>
+  <si>
+    <t>frequency of water return</t>
   </si>
 </sst>
 </file>
@@ -1931,4 +1965,96 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC9BDFCC-EE1E-8140-869D-9A85599D9AB0}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="48.1640625" customWidth="1"/>
+    <col min="3" max="3" width="15.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D1" s="3"/>
+    </row>
+    <row r="2" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="3"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D3" s="4"/>
+    </row>
+    <row r="4" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D5">
+        <v>860000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D6">
+        <v>7990000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B7" t="s">
+        <v>105</v>
+      </c>
+      <c r="C7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D7">
+        <v>3.4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>